<commit_message>
Complete FastAPI backend for Nifty100 Investment Analytics
</commit_message>
<xml_diff>
--- a/output/valuation_summary.xlsx
+++ b/output/valuation_summary.xlsx
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="I2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="b">
         <v>0</v>
@@ -739,11 +739,11 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="b">
         <v>0</v>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="I10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="b">
         <v>0</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="I12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="b">
         <v>0</v>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="I14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" t="b">
         <v>0</v>
@@ -1358,11 +1358,11 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J21" t="b">
         <v>0</v>
@@ -1406,7 +1406,7 @@
         </is>
       </c>
       <c r="I22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J22" t="b">
         <v>0</v>
@@ -1450,7 +1450,7 @@
         </is>
       </c>
       <c r="I23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J23" t="b">
         <v>0</v>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="I27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J27" t="b">
         <v>0</v>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="I33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J33" t="b">
         <v>0</v>
@@ -2151,11 +2151,11 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J39" t="b">
         <v>0</v>
@@ -2284,11 +2284,11 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="b">
         <v>0</v>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="b">
         <v>0</v>
@@ -2597,7 +2597,7 @@
         </is>
       </c>
       <c r="I49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" t="b">
         <v>0</v>
@@ -2642,7 +2642,7 @@
         </is>
       </c>
       <c r="I50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" t="b">
         <v>0</v>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="I51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J51" t="b">
         <v>0</v>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="I53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J53" t="b">
         <v>0</v>
@@ -3036,11 +3036,11 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I59" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J59" t="b">
         <v>0</v>
@@ -3124,11 +3124,11 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I61" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J61" t="b">
         <v>0</v>
@@ -3168,11 +3168,11 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I62" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J62" t="b">
         <v>0</v>
@@ -3393,7 +3393,7 @@
         </is>
       </c>
       <c r="I67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J67" t="b">
         <v>0</v>
@@ -3566,11 +3566,11 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="b">
         <v>0</v>
@@ -3610,11 +3610,11 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I72" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" t="b">
         <v>0</v>
@@ -3656,7 +3656,7 @@
         </is>
       </c>
       <c r="I73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J73" t="b">
         <v>0</v>
@@ -3740,11 +3740,11 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J75" t="b">
         <v>0</v>
@@ -4136,7 +4136,7 @@
         </is>
       </c>
       <c r="I84" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J84" t="b">
         <v>0</v>
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="I87" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J87" t="b">
         <v>0</v>
@@ -4359,7 +4359,7 @@
         </is>
       </c>
       <c r="I89" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J89" t="b">
         <v>0</v>
@@ -4399,11 +4399,11 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I90" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J90" t="b">
         <v>0</v>
@@ -4443,11 +4443,11 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Overvalued</t>
+          <t>Fairly Valued</t>
         </is>
       </c>
       <c r="I91" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91" t="b">
         <v>0</v>
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="I92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92" t="b">
         <v>0</v>
@@ -4535,7 +4535,7 @@
         </is>
       </c>
       <c r="I93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J93" t="b">
         <v>1</v>

</xml_diff>